<commit_message>
Lab4.2: robustness test project + complete Excel report
</commit_message>
<xml_diff>
--- a/Lab4_BVT.xlsx
+++ b/Lab4_BVT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pheerapat/Desktop/SaiWork/StudyKKU/SQA/Lab/Lab4/workspeac/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3955418-1971-AA49-8B6C-A86ABD8FB414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E42750A-D232-8A4F-8872-95BF6231BEC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16980" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,37 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="136">
+  <si>
+    <t>Test Strategy</t>
+  </si>
+  <si>
+    <t>No. of Test Cases</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>No run</t>
+  </si>
+  <si>
+    <t>Block</t>
+  </si>
+  <si>
+    <t>Remark / Defect ID</t>
+  </si>
+  <si>
+    <t>Normal Boundary Value Testing</t>
+  </si>
+  <si>
+    <t>Robustness Testing</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
   <si>
     <t>Test Case Design and Test Results</t>
   </si>
@@ -115,9 +145,6 @@
     <t>0</t>
   </si>
   <si>
-    <t>Pass</t>
-  </si>
-  <si>
     <t>TC002</t>
   </si>
   <si>
@@ -181,9 +208,6 @@
     <t>TC012</t>
   </si>
   <si>
-    <t>Fail</t>
-  </si>
-  <si>
     <t>TC013</t>
   </si>
   <si>
@@ -304,39 +328,45 @@
     <t>15 -&gt; EXCELLENT</t>
   </si>
   <si>
-    <t>Test Strategy</t>
-  </si>
-  <si>
-    <t>No. of Test Cases</t>
-  </si>
-  <si>
-    <t>No run</t>
-  </si>
-  <si>
-    <t>Block</t>
-  </si>
-  <si>
-    <t>Remark / Defect ID</t>
-  </si>
-  <si>
-    <t>Normal Boundary Value Testing</t>
-  </si>
-  <si>
-    <t>DEF-01 (VO2 decimal gap)</t>
-  </si>
-  <si>
-    <t>Robustness Testing</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
     <t>Lab 4.2</t>
   </si>
   <si>
     <t>Functional testing - Robustness Testing</t>
   </si>
   <si>
+    <t>Total = 10 -&gt; STANDARD</t>
+  </si>
+  <si>
+    <t>10 -&gt; STANDARD</t>
+  </si>
+  <si>
+    <t>IllegalArgumentException</t>
+  </si>
+  <si>
+    <t>throws</t>
+  </si>
+  <si>
+    <t>Total = 7 -&gt; STANDARD</t>
+  </si>
+  <si>
+    <t>7 -&gt; STANDARD</t>
+  </si>
+  <si>
+    <t>No upper bound -&gt; no throw, 5</t>
+  </si>
+  <si>
+    <t>no throw, 5</t>
+  </si>
+  <si>
+    <t>Pass*</t>
+  </si>
+  <si>
+    <t>Total = 8 -&gt; STANDARD</t>
+  </si>
+  <si>
+    <t>8 -&gt; STANDARD</t>
+  </si>
+  <si>
     <t>No</t>
   </si>
   <si>
@@ -383,13 +413,31 @@
   </si>
   <si>
     <t>VO2 ทศนิยมในช่วง (30,31),(40,41),(50,51) คืน 5 คะแนน เช่น 30.5 -&gt; 5 (ควรได้ 1) เพราะ else กว้างเกินไป (TC012-TC014)</t>
+  </si>
+  <si>
+    <t>DEF-02</t>
+  </si>
+  <si>
+    <t>VO2 Max และ HRR ไม่มีการ validate ขอบบน</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>VO2=91, HRR=61 (หรือค่ามหาศาล) ไม่ถูก reject คืน 5 เพราะ validateInputs เช็คแค่ค่าติดลบ ควรยืนยันกับสเปกว่าต้องมีเพดานบนไหม (TC007, TC019)</t>
+  </si>
+  <si>
+    <t>Robustness/DEF-02</t>
+  </si>
+  <si>
+    <t>Normal/DEF-01</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -448,6 +496,12 @@
       <color rgb="FFFF0000"/>
       <name val="TH SarabunPSK"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color rgb="FF0563C1"/>
+      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="7">
@@ -592,7 +646,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -634,11 +688,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -647,6 +696,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -665,7 +715,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
@@ -1010,36 +1071,36 @@
     <col min="2" max="2" width="17.1640625" style="1" customWidth="1"/>
     <col min="3" max="6" width="9.1640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="21.83203125" style="1" customWidth="1"/>
-    <col min="8" max="9" width="9.1640625" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.1640625" style="1"/>
+    <col min="8" max="11" width="9.1640625" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="56" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="13" t="s">
-        <v>93</v>
+        <v>0</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>94</v>
+        <v>1</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>95</v>
+        <v>4</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>96</v>
+        <v>5</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>97</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>98</v>
+        <v>7</v>
       </c>
       <c r="B3" s="3">
         <v>33</v>
@@ -1056,52 +1117,68 @@
       <c r="F3" s="3">
         <v>0</v>
       </c>
-      <c r="G3" s="17" t="s">
-        <v>99</v>
+      <c r="G3" s="30" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
+        <v>8</v>
+      </c>
+      <c r="B4" s="3">
+        <v>19</v>
+      </c>
+      <c r="C4" s="3">
+        <v>19</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3">
+        <v>0</v>
+      </c>
+      <c r="G4" s="31" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A6" s="21" t="s">
-        <v>101</v>
-      </c>
-      <c r="B6" s="6">
-        <v>33</v>
-      </c>
-      <c r="C6" s="18">
-        <v>30</v>
-      </c>
-      <c r="D6" s="19">
+      <c r="A6" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="3">
+        <v>52</v>
+      </c>
+      <c r="C6" s="32">
+        <v>49</v>
+      </c>
+      <c r="D6" s="33">
         <v>3</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="3">
         <v>0</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="3">
         <v>0</v>
       </c>
-      <c r="G6" s="20"/>
+      <c r="G6" s="17"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G3" location="'Normal'!A20" display="DEF-01 (VO2 decimal gap)" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="G4" location="'Robustness'!A15" display="DEF-02 (VO2/HRR no upper bound)" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1120,35 +1197,35 @@
     <col min="11" max="11" width="15.33203125" style="1" customWidth="1"/>
     <col min="12" max="12" width="10.83203125" style="1" customWidth="1"/>
     <col min="13" max="13" width="16.5" style="1" customWidth="1"/>
-    <col min="14" max="15" width="10.83203125" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="10.83203125" style="1"/>
+    <col min="14" max="17" width="10.83203125" style="1" customWidth="1"/>
+    <col min="18" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A1" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="26"/>
+      <c r="A1" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="24"/>
       <c r="J1" s="2"/>
       <c r="K1" s="8" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="G2" s="4"/>
       <c r="J2" s="3" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="K2" s="6">
         <v>-1</v>
@@ -1162,22 +1239,22 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
+        <v>15</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
       <c r="F3" s="5" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="K3" s="6">
         <v>0</v>
@@ -1191,22 +1268,22 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="27" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
+        <v>20</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
       <c r="F4" s="5" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="K4" s="6">
         <v>1</v>
@@ -1220,22 +1297,22 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="26"/>
+        <v>25</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="24"/>
       <c r="F5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="32">
+        <v>27</v>
+      </c>
+      <c r="G5" s="21">
         <v>46223</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="K5" s="6">
         <v>45</v>
@@ -1249,7 +1326,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="J6" s="3" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="K6" s="6">
         <v>89</v>
@@ -1262,25 +1339,25 @@
       </c>
     </row>
     <row r="7" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="25"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="G7" s="30" t="s">
-        <v>24</v>
+      <c r="A7" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="23"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="28" t="s">
+        <v>34</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="K7" s="6">
         <v>90</v>
@@ -1293,21 +1370,21 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A8" s="29"/>
+      <c r="A8" s="27"/>
       <c r="B8" s="8" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
+        <v>13</v>
+      </c>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
       <c r="J8" s="3" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="K8" s="6">
         <v>91</v>
@@ -1321,7 +1398,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" s="6" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="B9" s="6">
         <v>0</v>
@@ -1333,18 +1410,18 @@
         <v>20</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" s="6" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B10" s="6">
         <v>24.9</v>
@@ -1356,18 +1433,18 @@
         <v>20</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" s="6" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B11" s="6">
         <v>25</v>
@@ -1379,13 +1456,13 @@
         <v>20</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
@@ -1394,7 +1471,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" s="6" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B12" s="6">
         <v>30</v>
@@ -1406,13 +1483,13 @@
         <v>20</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
@@ -1421,7 +1498,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" s="6" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="B13" s="6">
         <v>31</v>
@@ -1433,13 +1510,13 @@
         <v>20</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
@@ -1448,7 +1525,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" s="6" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="B14" s="6">
         <v>40</v>
@@ -1460,13 +1537,13 @@
         <v>20</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
@@ -1475,7 +1552,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" s="6" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="B15" s="6">
         <v>41</v>
@@ -1487,13 +1564,13 @@
         <v>20</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
@@ -1502,7 +1579,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" s="6" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="B16" s="6">
         <v>50</v>
@@ -1514,13 +1591,13 @@
         <v>20</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
@@ -1529,7 +1606,7 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" s="6" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="B17" s="6">
         <v>51</v>
@@ -1541,19 +1618,19 @@
         <v>20</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J17" s="2"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" s="6" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="B18" s="6">
         <v>60</v>
@@ -1565,13 +1642,13 @@
         <v>20</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
@@ -1580,7 +1657,7 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" s="6" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="B19" s="6">
         <v>61</v>
@@ -1592,18 +1669,18 @@
         <v>20</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" s="6" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="B20" s="6">
         <v>30.5</v>
@@ -1615,18 +1692,18 @@
         <v>20</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>52</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" s="6" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="B21" s="6">
         <v>40.5</v>
@@ -1638,13 +1715,13 @@
         <v>20</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
@@ -1653,7 +1730,7 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" s="6" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B22" s="6">
         <v>50.5</v>
@@ -1665,13 +1742,13 @@
         <v>20</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
@@ -1680,7 +1757,7 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" s="6" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="B23" s="6">
         <v>45</v>
@@ -1692,13 +1769,13 @@
         <v>20</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
@@ -1707,7 +1784,7 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" s="6" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="B24" s="6">
         <v>45</v>
@@ -1719,13 +1796,13 @@
         <v>20</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
@@ -1734,7 +1811,7 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" s="6" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B25" s="6">
         <v>45</v>
@@ -1746,13 +1823,13 @@
         <v>20</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
@@ -1761,7 +1838,7 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" s="6" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="B26" s="6">
         <v>45</v>
@@ -1773,13 +1850,13 @@
         <v>20</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
@@ -1788,7 +1865,7 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27" s="6" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="B27" s="6">
         <v>45</v>
@@ -1800,19 +1877,19 @@
         <v>20</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J27" s="2"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A28" s="6" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="B28" s="6">
         <v>45</v>
@@ -1824,13 +1901,13 @@
         <v>20</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
@@ -1839,7 +1916,7 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A29" s="6" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="B29" s="6">
         <v>45</v>
@@ -1851,18 +1928,18 @@
         <v>0</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A30" s="6" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="B30" s="6">
         <v>45</v>
@@ -1874,18 +1951,18 @@
         <v>11</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A31" s="6" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B31" s="6">
         <v>45</v>
@@ -1897,18 +1974,18 @@
         <v>12</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A32" s="6" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="B32" s="6">
         <v>45</v>
@@ -1920,18 +1997,18 @@
         <v>18</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A33" s="6" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="B33" s="6">
         <v>45</v>
@@ -1943,18 +2020,18 @@
         <v>19</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="6" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="B34" s="6">
         <v>45</v>
@@ -1966,18 +2043,18 @@
         <v>24</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="6" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="B35" s="6">
         <v>45</v>
@@ -1989,18 +2066,18 @@
         <v>25</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="6" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="B36" s="6">
         <v>20</v>
@@ -2012,18 +2089,18 @@
         <v>5</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="6" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="B37" s="6">
         <v>45</v>
@@ -2035,18 +2112,18 @@
         <v>5</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="6" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="B38" s="6">
         <v>20</v>
@@ -2058,18 +2135,18 @@
         <v>25</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="6" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="B39" s="6">
         <v>65</v>
@@ -2081,18 +2158,18 @@
         <v>5</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A40" s="6" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="B40" s="6">
         <v>45</v>
@@ -2104,18 +2181,18 @@
         <v>20</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" s="6" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="B41" s="6">
         <v>65</v>
@@ -2127,13 +2204,13 @@
         <v>25</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2159,194 +2236,280 @@
   <cols>
     <col min="1" max="1" width="19.83203125" style="1" customWidth="1"/>
     <col min="2" max="4" width="21.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="23.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="30.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.1640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="25.1640625" style="1" customWidth="1"/>
     <col min="8" max="10" width="10.83203125" style="1" customWidth="1"/>
     <col min="11" max="11" width="15.33203125" style="1" customWidth="1"/>
     <col min="12" max="12" width="10.83203125" style="1" customWidth="1"/>
     <col min="13" max="13" width="16.5" style="1" customWidth="1"/>
-    <col min="14" max="15" width="10.83203125" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="10.83203125" style="1"/>
+    <col min="14" max="17" width="10.83203125" style="1" customWidth="1"/>
+    <col min="18" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A1" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="26"/>
+      <c r="A1" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="24"/>
       <c r="J1" s="2"/>
       <c r="K1" s="8" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="G2" s="4"/>
       <c r="J2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
+        <v>14</v>
+      </c>
+      <c r="K2" s="6">
+        <v>-1</v>
+      </c>
+      <c r="L2" s="6">
+        <v>39</v>
+      </c>
+      <c r="M2" s="6">
+        <v>-1</v>
+      </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="27" t="s">
-        <v>102</v>
-      </c>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
+        <v>15</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
       <c r="F3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="6"/>
+        <v>17</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>18</v>
+      </c>
       <c r="J3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
+        <v>19</v>
+      </c>
+      <c r="K3" s="6">
+        <v>0</v>
+      </c>
+      <c r="L3" s="6">
+        <v>40</v>
+      </c>
+      <c r="M3" s="6">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="27" t="s">
-        <v>103</v>
-      </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
+        <v>20</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
       <c r="F4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="6"/>
+        <v>22</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>23</v>
+      </c>
       <c r="J4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
+        <v>24</v>
+      </c>
+      <c r="K4" s="6">
+        <v>1</v>
+      </c>
+      <c r="L4" s="6">
+        <v>41</v>
+      </c>
+      <c r="M4" s="6">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="26"/>
+        <v>25</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="24"/>
       <c r="F5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="6"/>
+        <v>27</v>
+      </c>
+      <c r="G5" s="21">
+        <v>46223</v>
+      </c>
       <c r="J5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
+        <v>28</v>
+      </c>
+      <c r="K5" s="6">
+        <v>45</v>
+      </c>
+      <c r="L5" s="6">
+        <v>70</v>
+      </c>
+      <c r="M5" s="6">
+        <v>20</v>
+      </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="J6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
+        <v>29</v>
+      </c>
+      <c r="K6" s="6">
+        <v>89</v>
+      </c>
+      <c r="L6" s="6">
+        <v>219</v>
+      </c>
+      <c r="M6" s="6">
+        <v>59</v>
+      </c>
     </row>
     <row r="7" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="25"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="G7" s="30" t="s">
-        <v>24</v>
+      <c r="A7" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="23"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="28" t="s">
+        <v>34</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
+        <v>35</v>
+      </c>
+      <c r="K7" s="6">
+        <v>90</v>
+      </c>
+      <c r="L7" s="6">
+        <v>220</v>
+      </c>
+      <c r="M7" s="6">
+        <v>60</v>
+      </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A8" s="29"/>
+      <c r="A8" s="27"/>
       <c r="B8" s="8" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
+        <v>13</v>
+      </c>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
       <c r="J8" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
+        <v>36</v>
+      </c>
+      <c r="K8" s="6">
+        <v>91</v>
+      </c>
+      <c r="L8" s="6">
+        <v>221</v>
+      </c>
+      <c r="M8" s="6">
+        <v>61</v>
+      </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
+        <v>37</v>
+      </c>
+      <c r="B9" s="6">
+        <v>45</v>
+      </c>
+      <c r="C9" s="6">
+        <v>70</v>
+      </c>
+      <c r="D9" s="6">
+        <v>20</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
+        <v>40</v>
+      </c>
+      <c r="B10" s="6">
+        <v>-1</v>
+      </c>
+      <c r="C10" s="6">
+        <v>70</v>
+      </c>
+      <c r="D10" s="6">
+        <v>20</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
+        <v>41</v>
+      </c>
+      <c r="B11" s="6">
+        <v>0</v>
+      </c>
+      <c r="C11" s="6">
+        <v>70</v>
+      </c>
+      <c r="D11" s="6">
+        <v>20</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
@@ -2354,14 +2517,26 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
+        <v>44</v>
+      </c>
+      <c r="B12" s="6">
+        <v>1</v>
+      </c>
+      <c r="C12" s="6">
+        <v>70</v>
+      </c>
+      <c r="D12" s="6">
+        <v>20</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
@@ -2369,14 +2544,26 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
+        <v>45</v>
+      </c>
+      <c r="B13" s="6">
+        <v>89</v>
+      </c>
+      <c r="C13" s="6">
+        <v>70</v>
+      </c>
+      <c r="D13" s="6">
+        <v>20</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
@@ -2384,14 +2571,26 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
+        <v>48</v>
+      </c>
+      <c r="B14" s="6">
+        <v>90</v>
+      </c>
+      <c r="C14" s="6">
+        <v>70</v>
+      </c>
+      <c r="D14" s="6">
+        <v>20</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
@@ -2399,14 +2598,26 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
+        <v>49</v>
+      </c>
+      <c r="B15" s="6">
+        <v>91</v>
+      </c>
+      <c r="C15" s="6">
+        <v>70</v>
+      </c>
+      <c r="D15" s="6">
+        <v>20</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>111</v>
+      </c>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
@@ -2414,14 +2625,26 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
+        <v>52</v>
+      </c>
+      <c r="B16" s="6">
+        <v>45</v>
+      </c>
+      <c r="C16" s="6">
+        <v>39</v>
+      </c>
+      <c r="D16" s="6">
+        <v>20</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
@@ -2429,26 +2652,50 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
+        <v>53</v>
+      </c>
+      <c r="B17" s="6">
+        <v>45</v>
+      </c>
+      <c r="C17" s="6">
+        <v>40</v>
+      </c>
+      <c r="D17" s="6">
+        <v>20</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="J17" s="2"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
+        <v>56</v>
+      </c>
+      <c r="B18" s="6">
+        <v>45</v>
+      </c>
+      <c r="C18" s="6">
+        <v>41</v>
+      </c>
+      <c r="D18" s="6">
+        <v>20</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -2456,36 +2703,72 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="B19" s="6">
+        <v>45</v>
+      </c>
+      <c r="C19" s="6">
+        <v>219</v>
+      </c>
+      <c r="D19" s="6">
+        <v>20</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
+        <v>60</v>
+      </c>
+      <c r="B20" s="6">
+        <v>45</v>
+      </c>
+      <c r="C20" s="6">
+        <v>220</v>
+      </c>
+      <c r="D20" s="6">
+        <v>20</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A21" s="22" t="s">
-        <v>53</v>
-      </c>
-      <c r="B21" s="22"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
+      <c r="A21" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" s="19">
+        <v>45</v>
+      </c>
+      <c r="C21" s="19">
+        <v>221</v>
+      </c>
+      <c r="D21" s="19">
+        <v>20</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
@@ -2493,14 +2776,26 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
+        <v>62</v>
+      </c>
+      <c r="B22" s="6">
+        <v>45</v>
+      </c>
+      <c r="C22" s="6">
+        <v>70</v>
+      </c>
+      <c r="D22" s="6">
+        <v>-1</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
@@ -2508,14 +2803,26 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
+        <v>63</v>
+      </c>
+      <c r="B23" s="6">
+        <v>45</v>
+      </c>
+      <c r="C23" s="6">
+        <v>70</v>
+      </c>
+      <c r="D23" s="6">
+        <v>0</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
@@ -2523,14 +2830,26 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
+        <v>65</v>
+      </c>
+      <c r="B24" s="6">
+        <v>45</v>
+      </c>
+      <c r="C24" s="6">
+        <v>70</v>
+      </c>
+      <c r="D24" s="6">
+        <v>1</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
@@ -2538,14 +2857,26 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
+        <v>66</v>
+      </c>
+      <c r="B25" s="6">
+        <v>45</v>
+      </c>
+      <c r="C25" s="6">
+        <v>70</v>
+      </c>
+      <c r="D25" s="6">
+        <v>59</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
@@ -2553,14 +2884,26 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B26" s="6">
+        <v>45</v>
+      </c>
+      <c r="C26" s="6">
+        <v>70</v>
+      </c>
+      <c r="D26" s="6">
         <v>60</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
+      <c r="E26" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>2</v>
+      </c>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
@@ -2568,14 +2911,26 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B27" s="6">
+        <v>45</v>
+      </c>
+      <c r="C27" s="6">
+        <v>70</v>
+      </c>
+      <c r="D27" s="6">
         <v>61</v>
       </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
+      <c r="E27" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>111</v>
+      </c>
       <c r="J27" s="2"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.45">
@@ -2602,46 +2957,46 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A2:K3"/>
+  <dimension ref="A2:K4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="27" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="2" width="10.83203125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="4" width="10.83203125" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:11" ht="56" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="9" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.45">
@@ -2649,30 +3004,61 @@
         <v>1</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="D3" s="12">
         <v>46223</v>
       </c>
       <c r="E3" s="11"/>
       <c r="F3" s="6" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="J3" s="11"/>
       <c r="K3" s="11" t="s">
-        <v>119</v>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A4" s="11">
+        <v>2</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="D4" s="12">
+        <v>46223</v>
+      </c>
+      <c r="E4" s="11"/>
+      <c r="F4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>